<commit_message>
chore: update docs (publish)
</commit_message>
<xml_diff>
--- a/docs/pension_data_combined_2026-09-10.xlsx
+++ b/docs/pension_data_combined_2026-09-10.xlsx
@@ -1224,9 +1224,6 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="C48" t="n">
-        <v>1.144</v>
-      </c>
       <c r="D48" t="n">
         <v>4061522.58</v>
       </c>
@@ -1349,9 +1346,6 @@
         <is>
           <t>2026-09-10</t>
         </is>
-      </c>
-      <c r="C55" t="n">
-        <v>1.1874</v>
       </c>
       <c r="D55" t="n">
         <v>59159832.74</v>

</xml_diff>